<commit_message>
Audit excluded papers for hidden methods
</commit_message>
<xml_diff>
--- a/outputs/ICS-2026-计算传播学精选.xlsx
+++ b/outputs/ICS-2026-计算传播学精选.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="筛选说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="明确纳入" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="待全文确认" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="完整筛选记录" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="筛选说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明确纳入" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待全文确认" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整筛选记录" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'明确纳入'!$A$1:$Z$36</definedName>
@@ -7940,12 +7940,12 @@
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>摘要未显示计算方法或与计算传播相关的在线实验。</t>
+          <t>全文显示为荷兰代表性样本的预注册横截面在线问卷（n=2,196），使用 EFA、CFA、SEM 和调节分析；没有计算传播方法或实验操控。</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -8302,12 +8302,12 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>访谈、民族志、批判分析或其他质性方法；未使用计算方法。</t>
+          <t>全文以 Kiwi Farms 的公开帖文、平台文件与新闻材料重建平台迁移过程，采用质性案例分析；没有计算分析。</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -8424,12 +8424,12 @@
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>传统调查、面板或一般统计分析；摘要未显示计算方法或明确的在线实验。</t>
+          <t>全文显示为 Prolific 横截面在线问卷（n=375）与 PLS-SEM；没有实验操控或计算传播方法。</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -9160,12 +9160,12 @@
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>传统调查、面板或一般统计分析；摘要未显示计算方法或明确的在线实验。</t>
+          <t>全文显示为瑞典四波面板问卷（n=3,530），使用 RI-CLPM 与 LGCM；属于传统纵向调查分析。</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -12876,12 +12876,12 @@
       <c r="E61" s="2" t="inlineStr"/>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>传统调查、面板或一般统计分析；摘要未显示计算方法或明确的在线实验。</t>
+          <t>全文显示为两次相互关联的在线调查；第二次核验任务由人工按量规评分，分析使用 t 检验、相关和 OLS，不是随机实验。</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr"/>
@@ -12998,12 +12998,12 @@
       <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>摘要未显示计算方法或与计算传播相关的在线实验。</t>
+          <t>出版方页面标明该文为书评，不是经验研究论文。</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -16108,12 +16108,12 @@
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>摘要未显示计算方法或与计算传播相关的在线实验。</t>
+          <t>全文虽查询 Stack Exchange Data Dumps，但只用查询取得讨论串，核心材料缩减为 22 个线程并作溯因式质性分析；没有计算分析。</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17632,12 +17632,12 @@
       <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>访谈、民族志、批判分析或其他质性方法；未使用计算方法。</t>
+          <t>全文使用 Wakoopa 数字踪迹制作个体访谈提示材料，核心证据来自 73 次访谈及反思式主题分析；踪迹没有进入计算建模。</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr"/>
@@ -19242,12 +19242,12 @@
       <c r="E112" s="2" t="inlineStr"/>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>理论、概念或政策讨论；没有计算性经验方法。</t>
+          <t>全文先人工核验 407 个短视频，再选取 22 个视频进行人工多模态编码和质性解释；没有自动化或计算多模态分析。</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr"/>
@@ -20116,12 +20116,12 @@
       <c r="E119" s="2" t="inlineStr"/>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>传统调查、面板或一般统计分析；摘要未显示计算方法或明确的在线实验。</t>
+          <t>全文为全国在线问卷（n=2,373），向受访者展示带标签的既有图片并询问是否见过；只随机了题项顺序，没有随机处理条件。</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr"/>
@@ -24502,12 +24502,12 @@
       <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>摘要明确或原表方法明确</t>
+          <t>出版方全文方法明确</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>传统调查、面板或一般统计分析；摘要未显示计算方法或明确的在线实验。</t>
+          <t>全文确认为 2×4 随机组间在线情境实验；但研究涉及 AI 生成性影像虐待及色情网站情境，按用户本轮主题选择不收录。</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr"/>

</xml_diff>